<commit_message>
The latest LaSPUR website was created during the first training session
</commit_message>
<xml_diff>
--- a/report/preview/data/tabular/step1/tabel_acuan_pola_RTRW.xlsx
+++ b/report/preview/data/tabular/step1/tabel_acuan_pola_RTRW.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/f_mahezs_landscapealliance_org/Documents/ICRAF/Project/Solusi/LaSPUR/Data/v1/tabular/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ICRAF\Kodingan\icraf-indonesia\LaSPUR\report\preview\data\tabular\step1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{025372DB-8306-4B00-BA4D-AB5C123CFA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DA11B83-BDB5-40F7-9FCF-B6CEB19317DA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{997A8C56-B8CC-46E6-9E96-F53F4B8E9D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30610" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1BFA0940-7D81-4733-8CD1-3BF9DB729499}"/>
+    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="8880" xr2:uid="{1BFA0940-7D81-4733-8CD1-3BF9DB729499}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -50,9 +50,6 @@
     <t>RTRW</t>
   </si>
   <si>
-    <t>Prioritas</t>
-  </si>
-  <si>
     <t>Kawasan yang Memberikan Perlindungan terhadap Kawasan Bawahannya</t>
   </si>
   <si>
@@ -111,6 +108,9 @@
   </si>
   <si>
     <t>Kawasan Transportasi</t>
+  </si>
+  <si>
+    <t>Acuan Pola</t>
   </si>
 </sst>
 </file>
@@ -484,13 +484,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26D338C0-1963-48B6-8275-D8B0D04470E6}">
   <dimension ref="A1:C23"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="68.265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="68.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -498,142 +498,142 @@
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -644,29 +644,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -677,67 +677,67 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C18">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C23">
         <v>0</v>

</xml_diff>